<commit_message>
The domain is getawaycollective.co - carry it everywhere it was assumed
.in was assumed in eight files; the real site is getawaycollective.co.
The live server 301s www to the apex, so the apex is canonical and
NEXT_PUBLIC_SITE_URL, robots, sitemap, both lead-email defaults, the two
mailto fallbacks and the five contact addresses in the legal corpus all
carry it now. Workbook D-11 is recorded as answered, with the remaining
cutover fact: the domain currently serves a GoDaddy Website Builder
page, so repointing DNS to Vercel replaces it immediately.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GC-BUILD-STATE.xlsx
+++ b/GC-BUILD-STATE.xlsx
@@ -2745,10 +2745,10 @@
     <t xml:space="preserve">D-11</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirm the production domain.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">getawaycollective.in is assumed throughout .env.example. Every share card and sitemap URL depends on it.</t>
+    <t xml:space="preserve">ANSWERED 1 Aug 2026: the domain is getawaycollective.co (www 301s to the apex). The code now carries it. REMAINING: the domain currently serves a GoDaddy Website Builder page — DNS must be repointed to Vercel at go-live, and the builder page retired.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set NEXT_PUBLIC_SITE_URL=https://getawaycollective.co in Vercel. Decide the cutover moment: repointing DNS replaces the current GoDaddy page immediately.</t>
   </si>
   <si>
     <t xml:space="preserve">D-12</t>
@@ -15063,7 +15063,7 @@
       </c>
       <c r="I14" s="24"/>
     </row>
-    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
         <v>888</v>
       </c>

</xml_diff>